<commit_message>
BESP inflation adjusted, BPHEVSP timeline adjustment
</commit_message>
<xml_diff>
--- a/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
+++ b/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-newyork\InputData\trans\BESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EA3AF9-C5EF-4122-A2A1-D556860E9E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2940344-BCC1-4554-825A-87598C722703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="59820" yWindow="870" windowWidth="21825" windowHeight="15060" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="285">
   <si>
     <t>BESP BAU EV Subsidy Percentage</t>
   </si>
@@ -892,24 +892,33 @@
   </si>
   <si>
     <t>which models will apply under the requirements.</t>
+  </si>
+  <si>
+    <t>Inflation adjustment (2020 to 2012 USD)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1163,38 +1172,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="38" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="38" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" pivotButton="1" applyBorder="1"/>
@@ -1210,22 +1220,20 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="6" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1236,9 +1244,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 6" xfId="1" xr:uid="{7CEF46FD-FB9E-4904-A7BB-434C50DF8E47}"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -1283,7 +1294,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44965.625803356481" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44965.671375694445" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:P47" sheet="2019 Sales"/>
   </cacheSource>
@@ -2642,7 +2653,7 @@
       <c r="B1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="41">
+      <c r="C1" s="39">
         <v>44819</v>
       </c>
       <c r="F1" s="3" t="s">
@@ -3066,7 +3077,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="43" t="s">
+      <c r="A40" s="41" t="s">
         <v>282</v>
       </c>
       <c r="B40" s="4"/>
@@ -3078,7 +3089,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="40" t="s">
+      <c r="A41" s="38" t="s">
         <v>283</v>
       </c>
       <c r="B41" s="4"/>
@@ -3117,7 +3128,12 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B45" s="4"/>
+      <c r="A45" s="53">
+        <v>0.88711067149387013</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>284</v>
+      </c>
       <c r="F45" s="5" t="s">
         <v>114</v>
       </c>
@@ -6260,7 +6276,7 @@
     </row>
     <row r="4" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="31"/>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="40" t="s">
         <v>281</v>
       </c>
     </row>
@@ -6506,7 +6522,10 @@
     <row r="25" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31"/>
-      <c r="B26" s="31"/>
+      <c r="B26" s="31">
+        <f>C23*About!A45</f>
+        <v>1774.2213429877402</v>
+      </c>
       <c r="C26" s="31"/>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -6964,11 +6983,11 @@
         <v>4745.8606136031603</v>
       </c>
       <c r="B33" s="12">
-        <f t="shared" ref="B33:AF33" si="2">(B3+D23)</f>
+        <f>(B3+C23)</f>
         <v>4745.8606136031594</v>
       </c>
       <c r="C33" s="12">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="C33:AF33" si="2">(C3+D23)</f>
         <v>4745.8606136031603</v>
       </c>
       <c r="D33" s="12">
@@ -6989,7 +7008,7 @@
       </c>
       <c r="H33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="2"/>
@@ -11247,13 +11266,13 @@
       <c r="G24" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="H24" s="46">
+      <c r="H24" s="44">
         <v>175</v>
       </c>
-      <c r="I24" s="47">
+      <c r="I24" s="45">
         <v>210</v>
       </c>
-      <c r="J24" s="48">
+      <c r="J24" s="46">
         <v>45</v>
       </c>
       <c r="K24" s="8">
@@ -11271,13 +11290,13 @@
       <c r="G25" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="49">
+      <c r="H25" s="47">
         <v>997</v>
       </c>
-      <c r="I25" s="50">
+      <c r="I25" s="48">
         <v>1111</v>
       </c>
-      <c r="J25" s="51">
+      <c r="J25" s="49">
         <v>1147</v>
       </c>
       <c r="K25" s="8">
@@ -11295,13 +11314,13 @@
       <c r="G26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="H26" s="49">
+      <c r="H26" s="47">
         <v>72</v>
       </c>
-      <c r="I26" s="50">
+      <c r="I26" s="48">
         <v>87</v>
       </c>
-      <c r="J26" s="51">
+      <c r="J26" s="49">
         <v>33</v>
       </c>
       <c r="K26" s="8">
@@ -11319,13 +11338,13 @@
       <c r="G27" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="49">
+      <c r="H27" s="47">
         <v>557</v>
       </c>
-      <c r="I27" s="50">
+      <c r="I27" s="48">
         <v>573</v>
       </c>
-      <c r="J27" s="51">
+      <c r="J27" s="49">
         <v>611</v>
       </c>
       <c r="K27" s="8">
@@ -11343,13 +11362,13 @@
       <c r="G28" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H28" s="49">
+      <c r="H28" s="47">
         <v>2044</v>
       </c>
-      <c r="I28" s="50">
+      <c r="I28" s="48">
         <v>2430</v>
       </c>
-      <c r="J28" s="51">
+      <c r="J28" s="49">
         <v>3782</v>
       </c>
       <c r="K28" s="8">
@@ -11367,13 +11386,13 @@
       <c r="G29" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="H29" s="49">
+      <c r="H29" s="47">
         <v>1270</v>
       </c>
-      <c r="I29" s="50">
+      <c r="I29" s="48">
         <v>1281</v>
       </c>
-      <c r="J29" s="51">
+      <c r="J29" s="49">
         <v>1403</v>
       </c>
       <c r="K29" s="8">
@@ -11391,13 +11410,13 @@
       <c r="G30" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="H30" s="49">
+      <c r="H30" s="47">
         <v>111</v>
       </c>
-      <c r="I30" s="50">
+      <c r="I30" s="48">
         <v>173</v>
       </c>
-      <c r="J30" s="51">
+      <c r="J30" s="49">
         <v>256</v>
       </c>
       <c r="K30" s="8">
@@ -11415,13 +11434,13 @@
       <c r="G31" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="H31" s="49">
+      <c r="H31" s="47">
         <v>210</v>
       </c>
-      <c r="I31" s="50">
+      <c r="I31" s="48">
         <v>186</v>
       </c>
-      <c r="J31" s="51">
+      <c r="J31" s="49">
         <v>212</v>
       </c>
       <c r="K31" s="8">
@@ -11439,13 +11458,13 @@
       <c r="G32" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="H32" s="49">
+      <c r="H32" s="47">
         <v>309</v>
       </c>
-      <c r="I32" s="50">
+      <c r="I32" s="48">
         <v>517</v>
       </c>
-      <c r="J32" s="51">
+      <c r="J32" s="49">
         <v>240</v>
       </c>
       <c r="K32" s="8">
@@ -11463,13 +11482,13 @@
       <c r="G33" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="H33" s="49">
+      <c r="H33" s="47">
         <v>398</v>
       </c>
-      <c r="I33" s="50">
+      <c r="I33" s="48">
         <v>382</v>
       </c>
-      <c r="J33" s="51">
+      <c r="J33" s="49">
         <v>532</v>
       </c>
       <c r="K33" s="8">
@@ -11487,13 +11506,13 @@
       <c r="G34" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="49">
+      <c r="H34" s="47">
         <v>133</v>
       </c>
-      <c r="I34" s="50">
+      <c r="I34" s="48">
         <v>157</v>
       </c>
-      <c r="J34" s="51">
+      <c r="J34" s="49">
         <v>341</v>
       </c>
       <c r="K34" s="8">
@@ -11511,13 +11530,13 @@
       <c r="G35" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="H35" s="49">
+      <c r="H35" s="47">
         <v>717</v>
       </c>
-      <c r="I35" s="50">
+      <c r="I35" s="48">
         <v>654</v>
       </c>
-      <c r="J35" s="51">
+      <c r="J35" s="49">
         <v>1314</v>
       </c>
       <c r="K35" s="8">
@@ -11535,13 +11554,13 @@
       <c r="G36" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="H36" s="49">
+      <c r="H36" s="47">
         <v>215</v>
       </c>
-      <c r="I36" s="50">
+      <c r="I36" s="48">
         <v>255</v>
       </c>
-      <c r="J36" s="51">
+      <c r="J36" s="49">
         <v>310</v>
       </c>
       <c r="K36" s="8">
@@ -11559,11 +11578,11 @@
       <c r="G37" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="49"/>
-      <c r="I37" s="50">
+      <c r="H37" s="47"/>
+      <c r="I37" s="48">
         <v>27</v>
       </c>
-      <c r="J37" s="51">
+      <c r="J37" s="49">
         <v>52</v>
       </c>
       <c r="K37" s="8">
@@ -11581,13 +11600,13 @@
       <c r="G38" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="H38" s="49">
+      <c r="H38" s="47">
         <v>8000</v>
       </c>
-      <c r="I38" s="50">
+      <c r="I38" s="48">
         <v>7275</v>
       </c>
-      <c r="J38" s="51">
+      <c r="J38" s="49">
         <v>14625</v>
       </c>
       <c r="K38" s="8">
@@ -11605,13 +11624,13 @@
       <c r="G39" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="H39" s="49">
+      <c r="H39" s="47">
         <v>1123</v>
       </c>
-      <c r="I39" s="50">
+      <c r="I39" s="48">
         <v>1205</v>
       </c>
-      <c r="J39" s="51">
+      <c r="J39" s="49">
         <v>1820</v>
       </c>
       <c r="K39" s="8">
@@ -11629,13 +11648,13 @@
       <c r="G40" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="H40" s="49">
+      <c r="H40" s="47">
         <v>220</v>
       </c>
-      <c r="I40" s="50">
+      <c r="I40" s="48">
         <v>250</v>
       </c>
-      <c r="J40" s="51">
+      <c r="J40" s="49">
         <v>335</v>
       </c>
       <c r="K40" s="8">
@@ -11653,13 +11672,13 @@
       <c r="G41" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="H41" s="52">
+      <c r="H41" s="50">
         <v>164</v>
       </c>
-      <c r="I41" s="53">
+      <c r="I41" s="51">
         <v>118</v>
       </c>
-      <c r="J41" s="54">
+      <c r="J41" s="52">
         <v>581</v>
       </c>
       <c r="K41" s="8">
@@ -20383,7 +20402,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="42" t="s">
         <v>262</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -20397,7 +20416,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="45"/>
+      <c r="A2" s="43"/>
       <c r="B2" s="8" t="s">
         <v>266</v>
       </c>
@@ -20409,7 +20428,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="45"/>
+      <c r="A3" s="43"/>
       <c r="C3" s="8">
         <v>200000</v>
       </c>
@@ -20418,7 +20437,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="45"/>
+      <c r="A4" s="43"/>
       <c r="D4" s="8">
         <v>200000</v>
       </c>
@@ -21775,144 +21794,144 @@
       <c r="A2" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="B2" s="38">
+      <c r="B2" s="54">
         <f>C2</f>
-        <v>4745.8606136031603</v>
-      </c>
-      <c r="C2" s="38">
+        <v>4210.1035957498098</v>
+      </c>
+      <c r="C2" s="54">
         <f>D2</f>
-        <v>4745.8606136031603</v>
-      </c>
-      <c r="D2" s="38">
+        <v>4210.1035957498098</v>
+      </c>
+      <c r="D2" s="54">
         <f>E2</f>
-        <v>4745.8606136031603</v>
-      </c>
-      <c r="E2" s="39">
-        <f>Data!A33</f>
-        <v>4745.8606136031603</v>
-      </c>
-      <c r="F2" s="39">
-        <f>Data!B33</f>
-        <v>4745.8606136031594</v>
-      </c>
-      <c r="G2" s="39">
-        <f>Data!C33</f>
-        <v>4745.8606136031603</v>
-      </c>
-      <c r="H2" s="39">
-        <f>Data!D33</f>
-        <v>3913.0458308533107</v>
-      </c>
-      <c r="I2" s="39">
-        <f>Data!E33</f>
-        <v>2000</v>
-      </c>
-      <c r="J2" s="39">
-        <f>Data!F33</f>
-        <v>2000</v>
-      </c>
-      <c r="K2" s="39">
-        <f>Data!G33</f>
-        <v>2000</v>
-      </c>
-      <c r="L2" s="39">
-        <f>Data!H33</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="39">
-        <f>Data!I33</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="39">
-        <f>Data!J33</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="39">
-        <f>Data!K33</f>
-        <v>0</v>
-      </c>
-      <c r="P2" s="39">
-        <f>Data!L33</f>
-        <v>0</v>
-      </c>
-      <c r="Q2" s="39">
-        <f>Data!M33</f>
-        <v>0</v>
-      </c>
-      <c r="R2" s="39">
-        <f>Data!N33</f>
-        <v>0</v>
-      </c>
-      <c r="S2" s="39">
-        <f>Data!O33</f>
-        <v>0</v>
-      </c>
-      <c r="T2" s="39">
-        <f>Data!P33</f>
-        <v>0</v>
-      </c>
-      <c r="U2" s="39">
-        <f>Data!Q33</f>
-        <v>0</v>
-      </c>
-      <c r="V2" s="39">
-        <f>Data!R33</f>
-        <v>0</v>
-      </c>
-      <c r="W2" s="39">
-        <f>Data!S33</f>
-        <v>0</v>
-      </c>
-      <c r="X2" s="39">
-        <f>Data!T33</f>
-        <v>0</v>
-      </c>
-      <c r="Y2" s="39">
-        <f>Data!U33</f>
-        <v>0</v>
-      </c>
-      <c r="Z2" s="39">
-        <f>Data!V33</f>
-        <v>0</v>
-      </c>
-      <c r="AA2" s="39">
-        <f>Data!W33</f>
-        <v>0</v>
-      </c>
-      <c r="AB2" s="39">
-        <f>Data!X33</f>
-        <v>0</v>
-      </c>
-      <c r="AC2" s="39">
-        <f>Data!Y33</f>
-        <v>0</v>
-      </c>
-      <c r="AD2" s="39">
-        <f>Data!Z33</f>
-        <v>0</v>
-      </c>
-      <c r="AE2" s="39">
-        <f>Data!AA33</f>
-        <v>0</v>
-      </c>
-      <c r="AF2" s="39">
-        <f>Data!AB33</f>
-        <v>0</v>
-      </c>
-      <c r="AG2" s="39">
-        <f>Data!AC33</f>
-        <v>0</v>
-      </c>
-      <c r="AH2" s="39">
-        <f>Data!AD33</f>
-        <v>0</v>
-      </c>
-      <c r="AI2" s="39">
-        <f>Data!AE33</f>
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="39">
-        <f>Data!AF33</f>
+        <v>4210.1035957498098</v>
+      </c>
+      <c r="E2" s="12">
+        <f>Data!A33*About!$A45</f>
+        <v>4210.1035957498098</v>
+      </c>
+      <c r="F2" s="12">
+        <f>Data!B33*About!$A45</f>
+        <v>4210.1035957498088</v>
+      </c>
+      <c r="G2" s="12">
+        <f>Data!C33*About!$A45</f>
+        <v>4210.1035957498098</v>
+      </c>
+      <c r="H2" s="12">
+        <f>Data!D33*About!$A45</f>
+        <v>3471.3047145945693</v>
+      </c>
+      <c r="I2" s="12">
+        <f>Data!E33*About!$A45</f>
+        <v>1774.2213429877402</v>
+      </c>
+      <c r="J2" s="12">
+        <f>Data!F33*About!$A45</f>
+        <v>1774.2213429877402</v>
+      </c>
+      <c r="K2" s="12">
+        <f>Data!G33*About!$A45</f>
+        <v>1774.2213429877402</v>
+      </c>
+      <c r="L2" s="12">
+        <f>Data!H33*About!$A45</f>
+        <v>1774.2213429877402</v>
+      </c>
+      <c r="M2" s="12">
+        <f>Data!I33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="12">
+        <f>Data!J33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="12">
+        <f>Data!K33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="P2" s="12">
+        <f>Data!L33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="12">
+        <f>Data!M33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="12">
+        <f>Data!N33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="S2" s="12">
+        <f>Data!O33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="T2" s="12">
+        <f>Data!P33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="U2" s="12">
+        <f>Data!Q33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="V2" s="12">
+        <f>Data!R33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="W2" s="12">
+        <f>Data!S33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="X2" s="12">
+        <f>Data!T33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="12">
+        <f>Data!U33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="12">
+        <f>Data!V33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AA2" s="12">
+        <f>Data!W33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AB2" s="12">
+        <f>Data!X33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AC2" s="12">
+        <f>Data!Y33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AD2" s="12">
+        <f>Data!Z33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AE2" s="12">
+        <f>Data!AA33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AF2" s="12">
+        <f>Data!AB33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AG2" s="12">
+        <f>Data!AC33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AH2" s="12">
+        <f>Data!AD33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AI2" s="12">
+        <f>Data!AE33*About!$A45</f>
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="12">
+        <f>Data!AF33*About!$A45</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated to include entities of concern modeling from ICCT
</commit_message>
<xml_diff>
--- a/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
+++ b/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-newyork\InputData\trans\BESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2940344-BCC1-4554-825A-87598C722703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C760352E-0896-480A-B28E-2B15059A9440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="59820" yWindow="870" windowWidth="21825" windowHeight="15060" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60855" yWindow="2610" windowWidth="21600" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId8"/>
+    <pivotCache cacheId="7" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1233,6 +1233,8 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1244,8 +1246,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1294,7 +1294,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44965.671375694445" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44993.391117476851" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:P47" sheet="2019 Sales"/>
   </cacheSource>
@@ -2191,127 +2191,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="19">
-        <item x="10"/>
-        <item x="5"/>
-        <item x="16"/>
-        <item x="6"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="15"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="13"/>
-        <item x="11"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="17"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="14"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="19">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G22:J41" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
@@ -2430,6 +2310,126 @@
     <dataField name="Sum of JAN" fld="3" baseField="0"/>
     <dataField name="Sum of FEB" fld="4" baseField="0"/>
     <dataField name="Sum of MAR" fld="5" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="19">
+        <item x="10"/>
+        <item x="5"/>
+        <item x="16"/>
+        <item x="6"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="15"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="13"/>
+        <item x="11"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="17"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="14"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="2019 U.S. EV SALES" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JAN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="FEB" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="APR" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="MAY" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUN" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="JUL" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="AUG" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="SEP" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="OCT" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="NOV" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="DEC" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="TOTAL" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="19">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of TOTAL" fld="15" showDataAs="percentOfCol" baseField="0" numFmtId="10"/>
   </dataFields>
   <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3128,7 +3128,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="53">
+      <c r="A45" s="42">
         <v>0.88711067149387013</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -6185,72 +6185,95 @@
         <v>1913.0458308533109</v>
       </c>
       <c r="E3" s="11">
-        <v>0</v>
+        <f>BAU!G92</f>
+        <v>1531.9111519939402</v>
       </c>
       <c r="F3" s="11">
-        <v>0</v>
+        <f>BAU!H92</f>
+        <v>1131.4322818029341</v>
       </c>
       <c r="G3" s="11">
-        <v>0</v>
+        <f>BAU!I92</f>
+        <v>933.18813916995919</v>
       </c>
       <c r="H3" s="11">
-        <v>0</v>
+        <f>BAU!J92</f>
+        <v>933.18813916995953</v>
       </c>
       <c r="I3" s="11">
-        <v>0</v>
+        <f>BAU!K92</f>
+        <v>744.00735890914916</v>
       </c>
       <c r="J3" s="11">
-        <v>0</v>
+        <f>BAU!L92</f>
+        <v>744.00735890914984</v>
       </c>
       <c r="K3" s="11">
-        <v>0</v>
+        <f>BAU!M92</f>
+        <v>621.92251501542137</v>
       </c>
       <c r="L3" s="11">
-        <v>0</v>
+        <f>BAU!N92</f>
+        <v>240.24673989502756</v>
       </c>
       <c r="M3" s="11">
-        <v>0</v>
+        <f>BAU!O92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="N3" s="11">
-        <v>0</v>
+        <f>BAU!P92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="O3" s="11">
-        <v>0</v>
+        <f>BAU!Q92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="P3" s="11">
-        <v>0</v>
+        <f>BAU!R92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q3" s="11">
-        <v>0</v>
+        <f>BAU!S92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="R3" s="11">
-        <v>0</v>
+        <f>BAU!T92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="S3" s="11">
-        <v>0</v>
+        <f>BAU!U92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="T3" s="11">
+        <f>BAU!V92</f>
         <v>0</v>
       </c>
       <c r="U3" s="11">
+        <f>BAU!W92</f>
         <v>0</v>
       </c>
       <c r="V3" s="11">
+        <f>BAU!X92</f>
         <v>0</v>
       </c>
       <c r="W3" s="11">
+        <f>BAU!Y92</f>
         <v>0</v>
       </c>
       <c r="X3" s="11">
+        <f>BAU!Z92</f>
         <v>0</v>
       </c>
       <c r="Y3" s="11">
+        <f>BAU!AA92</f>
         <v>0</v>
       </c>
       <c r="Z3" s="11">
+        <f>BAU!AB92</f>
         <v>0</v>
       </c>
       <c r="AA3" s="11">
+        <f>BAU!AC92</f>
         <v>0</v>
       </c>
       <c r="AB3" s="11">
@@ -6996,63 +7019,63 @@
       </c>
       <c r="E33" s="12">
         <f t="shared" si="2"/>
-        <v>2000</v>
+        <v>3531.9111519939402</v>
       </c>
       <c r="F33" s="12">
         <f t="shared" si="2"/>
-        <v>2000</v>
+        <v>3131.4322818029341</v>
       </c>
       <c r="G33" s="12">
         <f t="shared" si="2"/>
-        <v>2000</v>
+        <v>2933.188139169959</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="2"/>
-        <v>2000</v>
+        <v>2933.1881391699594</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>744.00735890914916</v>
       </c>
       <c r="J33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>744.00735890914984</v>
       </c>
       <c r="K33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>621.92251501542137</v>
       </c>
       <c r="L33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>240.24673989502756</v>
       </c>
       <c r="M33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="N33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="O33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="P33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="R33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="S33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="T33" s="12">
         <f t="shared" si="2"/>
@@ -11266,13 +11289,13 @@
       <c r="G24" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="H24" s="44">
+      <c r="H24" s="46">
         <v>175</v>
       </c>
-      <c r="I24" s="45">
+      <c r="I24" s="47">
         <v>210</v>
       </c>
-      <c r="J24" s="46">
+      <c r="J24" s="48">
         <v>45</v>
       </c>
       <c r="K24" s="8">
@@ -11290,13 +11313,13 @@
       <c r="G25" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="47">
+      <c r="H25" s="49">
         <v>997</v>
       </c>
-      <c r="I25" s="48">
+      <c r="I25" s="50">
         <v>1111</v>
       </c>
-      <c r="J25" s="49">
+      <c r="J25" s="51">
         <v>1147</v>
       </c>
       <c r="K25" s="8">
@@ -11314,13 +11337,13 @@
       <c r="G26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="H26" s="47">
+      <c r="H26" s="49">
         <v>72</v>
       </c>
-      <c r="I26" s="48">
+      <c r="I26" s="50">
         <v>87</v>
       </c>
-      <c r="J26" s="49">
+      <c r="J26" s="51">
         <v>33</v>
       </c>
       <c r="K26" s="8">
@@ -11338,13 +11361,13 @@
       <c r="G27" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="47">
+      <c r="H27" s="49">
         <v>557</v>
       </c>
-      <c r="I27" s="48">
+      <c r="I27" s="50">
         <v>573</v>
       </c>
-      <c r="J27" s="49">
+      <c r="J27" s="51">
         <v>611</v>
       </c>
       <c r="K27" s="8">
@@ -11362,13 +11385,13 @@
       <c r="G28" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H28" s="47">
+      <c r="H28" s="49">
         <v>2044</v>
       </c>
-      <c r="I28" s="48">
+      <c r="I28" s="50">
         <v>2430</v>
       </c>
-      <c r="J28" s="49">
+      <c r="J28" s="51">
         <v>3782</v>
       </c>
       <c r="K28" s="8">
@@ -11386,13 +11409,13 @@
       <c r="G29" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="H29" s="47">
+      <c r="H29" s="49">
         <v>1270</v>
       </c>
-      <c r="I29" s="48">
+      <c r="I29" s="50">
         <v>1281</v>
       </c>
-      <c r="J29" s="49">
+      <c r="J29" s="51">
         <v>1403</v>
       </c>
       <c r="K29" s="8">
@@ -11410,13 +11433,13 @@
       <c r="G30" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="H30" s="47">
+      <c r="H30" s="49">
         <v>111</v>
       </c>
-      <c r="I30" s="48">
+      <c r="I30" s="50">
         <v>173</v>
       </c>
-      <c r="J30" s="49">
+      <c r="J30" s="51">
         <v>256</v>
       </c>
       <c r="K30" s="8">
@@ -11434,13 +11457,13 @@
       <c r="G31" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="H31" s="47">
+      <c r="H31" s="49">
         <v>210</v>
       </c>
-      <c r="I31" s="48">
+      <c r="I31" s="50">
         <v>186</v>
       </c>
-      <c r="J31" s="49">
+      <c r="J31" s="51">
         <v>212</v>
       </c>
       <c r="K31" s="8">
@@ -11458,13 +11481,13 @@
       <c r="G32" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="H32" s="47">
+      <c r="H32" s="49">
         <v>309</v>
       </c>
-      <c r="I32" s="48">
+      <c r="I32" s="50">
         <v>517</v>
       </c>
-      <c r="J32" s="49">
+      <c r="J32" s="51">
         <v>240</v>
       </c>
       <c r="K32" s="8">
@@ -11482,13 +11505,13 @@
       <c r="G33" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="H33" s="47">
+      <c r="H33" s="49">
         <v>398</v>
       </c>
-      <c r="I33" s="48">
+      <c r="I33" s="50">
         <v>382</v>
       </c>
-      <c r="J33" s="49">
+      <c r="J33" s="51">
         <v>532</v>
       </c>
       <c r="K33" s="8">
@@ -11506,13 +11529,13 @@
       <c r="G34" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="47">
+      <c r="H34" s="49">
         <v>133</v>
       </c>
-      <c r="I34" s="48">
+      <c r="I34" s="50">
         <v>157</v>
       </c>
-      <c r="J34" s="49">
+      <c r="J34" s="51">
         <v>341</v>
       </c>
       <c r="K34" s="8">
@@ -11530,13 +11553,13 @@
       <c r="G35" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="H35" s="47">
+      <c r="H35" s="49">
         <v>717</v>
       </c>
-      <c r="I35" s="48">
+      <c r="I35" s="50">
         <v>654</v>
       </c>
-      <c r="J35" s="49">
+      <c r="J35" s="51">
         <v>1314</v>
       </c>
       <c r="K35" s="8">
@@ -11554,13 +11577,13 @@
       <c r="G36" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="H36" s="47">
+      <c r="H36" s="49">
         <v>215</v>
       </c>
-      <c r="I36" s="48">
+      <c r="I36" s="50">
         <v>255</v>
       </c>
-      <c r="J36" s="49">
+      <c r="J36" s="51">
         <v>310</v>
       </c>
       <c r="K36" s="8">
@@ -11578,11 +11601,11 @@
       <c r="G37" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="47"/>
-      <c r="I37" s="48">
+      <c r="H37" s="49"/>
+      <c r="I37" s="50">
         <v>27</v>
       </c>
-      <c r="J37" s="49">
+      <c r="J37" s="51">
         <v>52</v>
       </c>
       <c r="K37" s="8">
@@ -11600,13 +11623,13 @@
       <c r="G38" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="H38" s="47">
+      <c r="H38" s="49">
         <v>8000</v>
       </c>
-      <c r="I38" s="48">
+      <c r="I38" s="50">
         <v>7275</v>
       </c>
-      <c r="J38" s="49">
+      <c r="J38" s="51">
         <v>14625</v>
       </c>
       <c r="K38" s="8">
@@ -11624,13 +11647,13 @@
       <c r="G39" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="H39" s="47">
+      <c r="H39" s="49">
         <v>1123</v>
       </c>
-      <c r="I39" s="48">
+      <c r="I39" s="50">
         <v>1205</v>
       </c>
-      <c r="J39" s="49">
+      <c r="J39" s="51">
         <v>1820</v>
       </c>
       <c r="K39" s="8">
@@ -11648,13 +11671,13 @@
       <c r="G40" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="H40" s="47">
+      <c r="H40" s="49">
         <v>220</v>
       </c>
-      <c r="I40" s="48">
+      <c r="I40" s="50">
         <v>250</v>
       </c>
-      <c r="J40" s="49">
+      <c r="J40" s="51">
         <v>335</v>
       </c>
       <c r="K40" s="8">
@@ -11672,13 +11695,13 @@
       <c r="G41" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="H41" s="50">
+      <c r="H41" s="52">
         <v>164</v>
       </c>
-      <c r="I41" s="51">
+      <c r="I41" s="53">
         <v>118</v>
       </c>
-      <c r="J41" s="52">
+      <c r="J41" s="54">
         <v>581</v>
       </c>
       <c r="K41" s="8">
@@ -20402,7 +20425,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>262</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -20416,7 +20439,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="43"/>
+      <c r="A2" s="45"/>
       <c r="B2" s="8" t="s">
         <v>266</v>
       </c>
@@ -20428,7 +20451,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="43"/>
+      <c r="A3" s="45"/>
       <c r="C3" s="8">
         <v>200000</v>
       </c>
@@ -20437,7 +20460,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
+      <c r="A4" s="45"/>
       <c r="D4" s="8">
         <v>200000</v>
       </c>
@@ -21794,15 +21817,15 @@
       <c r="A2" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="B2" s="54">
+      <c r="B2" s="43">
         <f>C2</f>
         <v>4210.1035957498098</v>
       </c>
-      <c r="C2" s="54">
+      <c r="C2" s="43">
         <f>D2</f>
         <v>4210.1035957498098</v>
       </c>
-      <c r="D2" s="54">
+      <c r="D2" s="43">
         <f>E2</f>
         <v>4210.1035957498098</v>
       </c>
@@ -21824,63 +21847,63 @@
       </c>
       <c r="I2" s="12">
         <f>Data!E33*About!$A45</f>
-        <v>1774.2213429877402</v>
+        <v>3133.1960737020327</v>
       </c>
       <c r="J2" s="12">
         <f>Data!F33*About!$A45</f>
-        <v>1774.2213429877402</v>
+        <v>2777.9269942477827</v>
       </c>
       <c r="K2" s="12">
         <f>Data!G33*About!$A45</f>
-        <v>1774.2213429877402</v>
+        <v>2602.0624997569175</v>
       </c>
       <c r="L2" s="12">
         <f>Data!H33*About!$A45</f>
-        <v>1774.2213429877402</v>
+        <v>2602.062499756918</v>
       </c>
       <c r="M2" s="12">
         <f>Data!I33*About!$A45</f>
-        <v>0</v>
+        <v>660.01686775827613</v>
       </c>
       <c r="N2" s="12">
         <f>Data!J33*About!$A45</f>
-        <v>0</v>
+        <v>660.0168677582767</v>
       </c>
       <c r="O2" s="12">
         <f>Data!K33*About!$A45</f>
-        <v>0</v>
+        <v>551.71409991248697</v>
       </c>
       <c r="P2" s="12">
         <f>Data!L33*About!$A45</f>
-        <v>0</v>
+        <v>213.12544675249106</v>
       </c>
       <c r="Q2" s="12">
         <f>Data!M33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="R2" s="12">
         <f>Data!N33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="S2" s="12">
         <f>Data!O33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="T2" s="12">
         <f>Data!P33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="U2" s="12">
         <f>Data!Q33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="V2" s="12">
         <f>Data!R33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="W2" s="12">
         <f>Data!S33*About!$A45</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="X2" s="12">
         <f>Data!T33*About!$A45</f>

</xml_diff>